<commit_message>
Update policies, imports and resource tables with enhanced permissions
</commit_message>
<xml_diff>
--- a/template_user.xlsx
+++ b/template_user.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="111">
   <si>
     <t>Nama</t>
   </si>
@@ -36,6 +36,9 @@
     <t>Department</t>
   </si>
   <si>
+    <t>Roles</t>
+  </si>
+  <si>
     <t xml:space="preserve">Aart van Wingerden</t>
   </si>
   <si>
@@ -48,6 +51,9 @@
     <t>Management</t>
   </si>
   <si>
+    <t xml:space="preserve">Super Admin</t>
+  </si>
+  <si>
     <t xml:space="preserve">Donny Seprana Marabunta</t>
   </si>
   <si>
@@ -75,6 +81,9 @@
     <t>Marketing</t>
   </si>
   <si>
+    <t>Manager</t>
+  </si>
+  <si>
     <t xml:space="preserve">Moh. Reyyan Puja Laksana</t>
   </si>
   <si>
@@ -99,6 +108,9 @@
     <t xml:space="preserve">Under Jr. Product Manager</t>
   </si>
   <si>
+    <t>Staff</t>
+  </si>
+  <si>
     <t xml:space="preserve">R. Hapsarendra Gunung Drajat</t>
   </si>
   <si>
@@ -124,6 +136,9 @@
   </si>
   <si>
     <t xml:space="preserve">Under RSM</t>
+  </si>
+  <si>
+    <t>Supervisor</t>
   </si>
   <si>
     <t xml:space="preserve">Resa Aydwi</t>
@@ -951,7 +966,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col customWidth="1" min="1" max="6" width="30.7109375"/>
+    <col customWidth="1" min="1" max="7" width="30.7109375"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -973,549 +988,639 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" s="1"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" s="5"/>
       <c r="F3" s="3" t="s">
-        <v>9</v>
+        <v>10</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4" s="4"/>
       <c r="F4" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="E6" s="4"/>
       <c r="F6" s="4" t="s">
-        <v>18</v>
+        <v>20</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C8" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="4" t="s">
+      <c r="F8" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>31</v>
+      <c r="G8" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E9" s="3" t="s">
+      <c r="G9" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="B10" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E10" s="3" t="s">
+      <c r="G10" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="D11" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="3" t="s">
+      <c r="G11" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="D12" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="E12" s="3" t="s">
+      <c r="G12" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="E13" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="E14" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="4" t="s">
         <v>30</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="11" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C17" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="E17" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D17" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>53</v>
-      </c>
       <c r="F17" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>31</v>
+        <v>35</v>
+      </c>
+      <c r="G18" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C19" s="9" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E19" s="4"/>
       <c r="F19" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="G19" s="4" t="s">
+        <v>21</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E20" s="4"/>
       <c r="F20" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="E21" s="4"/>
       <c r="F21" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="G21" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="11" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="E22" s="4"/>
       <c r="F22" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="E23" s="3"/>
       <c r="F23" s="4" t="s">
-        <v>64</v>
+        <v>69</v>
+      </c>
+      <c r="G23" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E24" s="3"/>
       <c r="F24" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="E25" s="5"/>
       <c r="F25" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="C26" s="9" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E26" s="4"/>
       <c r="F26" s="3" t="s">
-        <v>91</v>
+        <v>96</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E27" s="7"/>
       <c r="F27" s="7" t="s">
-        <v>95</v>
+        <v>100</v>
+      </c>
+      <c r="G27" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="C28" s="9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E28" s="4"/>
       <c r="F28" s="4" t="s">
-        <v>95</v>
+        <v>100</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="C29" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E29" s="4"/>
       <c r="F29" s="4" t="s">
-        <v>102</v>
+        <v>107</v>
+      </c>
+      <c r="G29" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B30" s="7" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="C30" s="9" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E30" s="4"/>
       <c r="F30" s="4" t="s">
-        <v>102</v>
+        <v>107</v>
+      </c>
+      <c r="G30" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>